<commit_message>
Add period reports, gender tracking, source of data, community fix
</commit_message>
<xml_diff>
--- a/kobo/YALL_MEAL_Indicator_Update.xlsx
+++ b/kobo/YALL_MEAL_Indicator_Update.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -505,12 +505,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Community (leave blank or choose 'Project-wide' if this isn't tied to one community)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -685,48 +685,48 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>obs_date</t>
+          <t>male</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Date of observation</t>
+          <t>Of that number, how many were male? (optional)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>instance('indicator')/root/item[name=${indicator}]/gender='yes'</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>today()</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>female</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GPS location (optional — tap to capture on site)</t>
+          <t>Of that number, how many were female? (optional)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -734,7 +734,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>instance('indicator')/root/item[name=${indicator}]/gender='yes'</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -743,44 +747,48 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>photo</t>
+          <t>obs_date</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Photo evidence (optional)</t>
+          <t>Date of observation</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>today()</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Notes / context (optional)</t>
+          <t>GPS location (optional — tap to capture on site)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -797,22 +805,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>select_one coordinator</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>photo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Recorded by</t>
+          <t>Photo evidence (optional)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -820,6 +828,60 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Notes / context (optional)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>select_one coordinator</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Recorded by</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -832,7 +894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -861,6 +923,11 @@
           <t>kind</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -880,6 +947,7 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -899,6 +967,7 @@
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -918,6 +987,7 @@
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -937,6 +1007,7 @@
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -960,6 +1031,7 @@
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -983,6 +1055,7 @@
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1006,6 +1079,7 @@
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1029,6 +1103,7 @@
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1052,6 +1127,7 @@
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1061,20 +1137,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>tormue</t>
+          <t>not_community_specific</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tormue</t>
+          <t>Project-wide (not tied to one community)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1084,12 +1161,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>yowee</t>
+          <t>tormue</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Yowee</t>
+          <t>Tormue</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1098,6 +1175,7 @@
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1107,20 +1185,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>kiliwu</t>
+          <t>yowee</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Kiliwu</t>
+          <t>Yowee</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1130,20 +1209,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>zolowo</t>
+          <t>not_community_specific</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Zolowo</t>
+          <t>Project-wide (not tied to one community)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1153,12 +1233,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>kponwansanyea_kpeteyea</t>
+          <t>kiliwu</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kponwansanyea-Kpeteyea</t>
+          <t>Kiliwu</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1167,6 +1247,7 @@
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1176,12 +1257,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>kpayaquelleh_new_town</t>
+          <t>zolowo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Kpayaquelleh New Town</t>
+          <t>Zolowo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1190,6 +1271,7 @@
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1199,12 +1281,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>yowee</t>
+          <t>kponwansanyea_kpeteyea</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Yowee</t>
+          <t>Kponwansanyea-Kpeteyea</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1213,6 +1295,7 @@
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1222,12 +1305,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>gbargonai</t>
+          <t>kpayaquelleh_new_town</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Gbargonai</t>
+          <t>Kpayaquelleh New Town</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1236,6 +1319,7 @@
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1245,12 +1329,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>david_deans_town</t>
+          <t>yowee</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>David Deans Town</t>
+          <t>Yowee</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1259,6 +1343,7 @@
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1268,20 +1353,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>kiliwu</t>
+          <t>gbargonai</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Kiliwu</t>
+          <t>Gbargonai</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1291,20 +1377,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>kponwansanyea_kpeteyea</t>
+          <t>david_deans_town</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Kponwansanyea-Kpeteyea</t>
+          <t>David Deans Town</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1314,20 +1401,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>kpayaquelleh_new_town</t>
+          <t>not_community_specific</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Kpayaquelleh New Town</t>
+          <t>Project-wide (not tied to one community)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1337,12 +1425,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>yowee</t>
+          <t>kiliwu</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Yowee</t>
+          <t>Kiliwu</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1351,6 +1439,7 @@
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1360,12 +1449,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>tormue</t>
+          <t>kponwansanyea_kpeteyea</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tormue</t>
+          <t>Kponwansanyea-Kpeteyea</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1374,114 +1463,103 @@
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>indicator</t>
+          <t>community</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>kpayaquelleh_new_town</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Women leaders trained in legal empowerment, water monitoring, evidence gathering (women leaders)</t>
+          <t>Kpayaquelleh New Town</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>uaf_women</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>indicator</t>
+          <t>community</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>yowee</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Community dialogue sessions conducted (sessions)</t>
+          <t>Yowee</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>uaf_women</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>indicator</t>
+          <t>community</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>tormue</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Shadow report published (reports)</t>
+          <t>Tormue</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>uaf_women</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>indicator</t>
+          <t>community</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>i4</t>
+          <t>not_community_specific</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Copies of shadow report disseminated (copies)</t>
+          <t>Project-wide (not tied to one community)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>uaf_women</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1491,12 +1569,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>i5</t>
+          <t>i1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Advocacy meetings held with decision-makers (meetings)</t>
+          <t>Women leaders trained in legal empowerment, water monitoring, evidence gathering (women leaders)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1507,6 +1585,11 @@
       <c r="E29" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1518,12 +1601,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>i6</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>New EPA investigations initiated from community-generated evidence (investigations)</t>
+          <t>Community dialogue sessions conducted (sessions)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1534,6 +1617,11 @@
       <c r="E30" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1545,12 +1633,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>i7</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Agroecology demonstration plots established (plots)</t>
+          <t>Shadow report published (reports)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1561,6 +1649,11 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1572,12 +1665,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>i8</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Women farmers trained in agroecological practices (women farmers)</t>
+          <t>Copies of shadow report disseminated (copies)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1588,6 +1681,11 @@
       <c r="E32" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1697,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>i9</t>
+          <t>i5</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Women farmers adopting at least 4 agroecological techniques (women farmers)</t>
+          <t>Advocacy meetings held with decision-makers (meetings)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1615,6 +1713,11 @@
       <c r="E33" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1626,12 +1729,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>i10</t>
+          <t>i6</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Radio awareness sessions aired (sessions)</t>
+          <t>New EPA investigations initiated from community-generated evidence (investigations)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1642,6 +1745,11 @@
       <c r="E34" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1653,12 +1761,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>i11</t>
+          <t>i7</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Social media content pieces produced (content pieces)</t>
+          <t>Agroecology demonstration plots established (plots)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1669,6 +1777,11 @@
       <c r="E35" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1680,12 +1793,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>i12</t>
+          <t>i8</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CSOs participating in the Rural Women Climate Justice Summit (organizations)</t>
+          <t>Women farmers trained in agroecological practices (women farmers)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1696,6 +1809,11 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1707,12 +1825,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>i13</t>
+          <t>i9</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Policy proposal tabled by coalition (proposals)</t>
+          <t>Women farmers adopting at least 4 agroecological techniques (women farmers)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1723,6 +1841,11 @@
       <c r="E37" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1734,12 +1857,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>i14</t>
+          <t>i10</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Organizations in the coalition tabling the policy proposal (organizations)</t>
+          <t>Radio awareness sessions aired (sessions)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1750,6 +1873,11 @@
       <c r="E38" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1761,22 +1889,27 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>i15</t>
+          <t>i11</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Agroecological demonstration sites established (sites)</t>
+          <t>Social media content pieces produced (content pieces)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1788,22 +1921,27 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>i16</t>
+          <t>i12</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Demonstration sites with soil and water conservation structures in place (sites)</t>
+          <t>CSOs participating in the Rural Women Climate Justice Summit (organizations)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1815,22 +1953,27 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>i17</t>
+          <t>i13</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Tool sheds and storage units constructed (sheds)</t>
+          <t>Policy proposal tabled by coalition (proposals)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1842,22 +1985,27 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>i18</t>
+          <t>i14</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Farmers trained in climate-smart agroecological practices (farmers)</t>
+          <t>Organizations in the coalition tabling the policy proposal (organizations)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1869,12 +2017,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>i19</t>
+          <t>i15</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Female participants among trained farmers (%)</t>
+          <t>Agroecological demonstration sites established (sites)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1884,7 +2032,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1896,12 +2049,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>i20</t>
+          <t>i16</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Trained farmers demonstrating knowledge of at least 3 techniques (%)</t>
+          <t>Demonstration sites with soil and water conservation structures in place (sites)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1911,7 +2064,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1923,12 +2081,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>i21</t>
+          <t>i17</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Trained farmers adopting at least 3 new practices (%)</t>
+          <t>Tool sheds and storage units constructed (sheds)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1938,7 +2096,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1950,12 +2113,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>i22</t>
+          <t>i18</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Vegetable crop varieties planted and harvested (varieties)</t>
+          <t>Farmers trained in climate-smart agroecological practices (farmers)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1966,6 +2129,11 @@
       <c r="E46" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1977,12 +2145,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>i23</t>
+          <t>i19</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Harvest consumed by participating households (%)</t>
+          <t>Female participants among trained farmers (%)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1993,6 +2161,11 @@
       <c r="E47" t="inlineStr">
         <is>
           <t>percent</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2004,12 +2177,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>i24</t>
+          <t>i20</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Harvest sold collectively (%)</t>
+          <t>Trained farmers demonstrating knowledge of at least 3 techniques (%)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2020,6 +2193,11 @@
       <c r="E48" t="inlineStr">
         <is>
           <t>percent</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2031,12 +2209,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>i25</t>
+          <t>i21</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Farmers completing agro-entrepreneurship training (farmers)</t>
+          <t>Trained farmers adopting at least 3 new practices (%)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2046,7 +2224,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2058,12 +2241,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>i26</t>
+          <t>i22</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Farmer groups maintaining financial records (groups)</t>
+          <t>Vegetable crop varieties planted and harvested (varieties)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2074,6 +2257,11 @@
       <c r="E50" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2085,12 +2273,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>i27</t>
+          <t>i23</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Farmer groups with an active susu fund (groups)</t>
+          <t>Harvest consumed by participating households (%)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2100,7 +2288,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2112,12 +2305,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>i28</t>
+          <t>i24</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Increase in average household income from produce sales (%)</t>
+          <t>Harvest sold collectively (%)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2127,7 +2320,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2139,12 +2337,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>i29</t>
+          <t>i25</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Farmer groups participating in final evaluation workshop (groups)</t>
+          <t>Farmers completing agro-entrepreneurship training (farmers)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2155,6 +2353,11 @@
       <c r="E53" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2166,12 +2369,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>i30</t>
+          <t>i26</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Written sustainability plans produced and adopted (plans)</t>
+          <t>Farmer groups maintaining financial records (groups)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2182,6 +2385,11 @@
       <c r="E54" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2193,22 +2401,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>i31</t>
+          <t>i27</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Formal partnership agreement signed with EPA (agreements)</t>
+          <t>Farmer groups with an active susu fund (groups)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2220,22 +2433,27 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>i32</t>
+          <t>i28</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Joint activities conducted with EPA (activities)</t>
+          <t>Increase in average household income from produce sales (%)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2247,22 +2465,27 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>i33</t>
+          <t>i29</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Community members trained on legal advocacy (people)</t>
+          <t>Farmer groups participating in final evaluation workshop (groups)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2274,22 +2497,27 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>i34</t>
+          <t>i30</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Trained community members demonstrating improved knowledge of land rights (%)</t>
+          <t>Written sustainability plans produced and adopted (plans)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2301,12 +2529,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>i35</t>
+          <t>i31</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Trained community members who know where to report environmental damage (%)</t>
+          <t>Formal partnership agreement signed with EPA (agreements)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2316,7 +2544,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2328,12 +2561,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>i36</t>
+          <t>i32</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Community members engaged in documented advocacy action post-training (people)</t>
+          <t>Joint activities conducted with EPA (activities)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2344,6 +2577,11 @@
       <c r="E60" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2355,12 +2593,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>i37</t>
+          <t>i33</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Community advocacy associations formed and active (associations)</t>
+          <t>Community members trained on legal advocacy (people)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2371,6 +2609,11 @@
       <c r="E61" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2382,12 +2625,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>i38</t>
+          <t>i34</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Active members across community advocacy associations (members)</t>
+          <t>Trained community members demonstrating improved knowledge of land rights (%)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2397,7 +2640,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2409,12 +2657,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>i39</t>
+          <t>i35</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Advocacy actions taken by association members (actions)</t>
+          <t>Trained community members who know where to report environmental damage (%)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2424,7 +2672,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2436,12 +2689,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>i40</t>
+          <t>i36</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Community members reached through association-led advocacy activities (people)</t>
+          <t>Community members engaged in documented advocacy action post-training (people)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2452,6 +2705,11 @@
       <c r="E64" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2463,12 +2721,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>i41</t>
+          <t>i37</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Miners trained on safe mining practices (miners)</t>
+          <t>Community advocacy associations formed and active (associations)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2479,6 +2737,11 @@
       <c r="E65" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2490,12 +2753,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>i42</t>
+          <t>i38</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Trained miners demonstrating improved knowledge of safety protocols (%)</t>
+          <t>Active members across community advocacy associations (members)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2505,7 +2768,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2517,12 +2785,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>i43</t>
+          <t>i39</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Trained miners reporting consistent PPE use post-training (%)</t>
+          <t>Advocacy actions taken by association members (actions)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2532,7 +2800,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2544,12 +2817,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>i44</t>
+          <t>i40</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Trained miners aware of mining laws and regulations (%)</t>
+          <t>Community members reached through association-led advocacy activities (people)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2559,7 +2832,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2571,12 +2849,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>i45</t>
+          <t>i41</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Miners who fill or cover pits after mining (%)</t>
+          <t>Miners trained on safe mining practices (miners)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2586,7 +2864,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2598,12 +2881,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>i46</t>
+          <t>i42</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Students reached through climate change workshops (students)</t>
+          <t>Trained miners demonstrating improved knowledge of safety protocols (%)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2613,7 +2896,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2625,12 +2913,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>i47</t>
+          <t>i43</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Schools participating in climate change workshops (schools)</t>
+          <t>Trained miners reporting consistent PPE use post-training (%)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2640,7 +2928,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2652,12 +2945,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>i48</t>
+          <t>i44</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Students demonstrating improved climate change knowledge (%)</t>
+          <t>Trained miners aware of mining laws and regulations (%)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2668,6 +2961,11 @@
       <c r="E72" t="inlineStr">
         <is>
           <t>percent</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2679,12 +2977,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>i49</t>
+          <t>i45</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Climate Justice Hub established and operational (hubs)</t>
+          <t>Miners who fill or cover pits after mining (%)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2694,7 +2992,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2706,12 +3009,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>i50</t>
+          <t>i46</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Community-led climate-sensitive projects initiated through the hub (projects)</t>
+          <t>Students reached through climate change workshops (students)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2722,6 +3025,11 @@
       <c r="E74" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2733,12 +3041,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>i51</t>
+          <t>i47</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Community members engaged through hub activities (people)</t>
+          <t>Schools participating in climate change workshops (schools)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2749,6 +3057,11 @@
       <c r="E75" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2760,12 +3073,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>i52</t>
+          <t>i48</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Training manuals developed (manuals)</t>
+          <t>Students demonstrating improved climate change knowledge (%)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2775,7 +3088,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2787,12 +3105,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>i53</t>
+          <t>i49</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Training sessions conducted using the developed manuals (%)</t>
+          <t>Climate Justice Hub established and operational (hubs)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2802,7 +3120,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2814,12 +3137,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>i54</t>
+          <t>i50</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Facilitators rating the training manuals as useful or highly useful (%)</t>
+          <t>Community-led climate-sensitive projects initiated through the hub (projects)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2829,7 +3152,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2841,22 +3169,27 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>i55</t>
+          <t>i51</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Women farmers participating in training (women farmers)</t>
+          <t>Community members engaged through hub activities (people)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2868,22 +3201,27 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>i56</t>
+          <t>i52</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Women farmers who know at least 3 climate-smart techniques (%)</t>
+          <t>Training manuals developed (manuals)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2895,22 +3233,27 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>i57</t>
+          <t>i53</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Women farmers applying at least 3 techniques on their farms (%)</t>
+          <t>Training sessions conducted using the developed manuals (%)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>percent</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2922,22 +3265,27 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>i58</t>
+          <t>i54</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Average crop yield increase (%)</t>
+          <t>Facilitators rating the training manuals as useful or highly useful (%)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2949,12 +3297,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>i59</t>
+          <t>i55</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Women-led agricultural groups legally registered (groups)</t>
+          <t>Women farmers participating in training (women farmers)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2965,6 +3313,11 @@
       <c r="E83" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2976,12 +3329,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>i60</t>
+          <t>i56</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Registered groups actively selling produce together (groups)</t>
+          <t>Women farmers who know at least 3 climate-smart techniques (%)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2991,7 +3344,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3003,12 +3361,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>i61</t>
+          <t>i57</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Average increase in group sales revenue (%)</t>
+          <t>Women farmers applying at least 3 techniques on their farms (%)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3018,7 +3376,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3030,12 +3393,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>i62</t>
+          <t>i58</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Average increase in household income (%)</t>
+          <t>Average crop yield increase (%)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3046,6 +3409,11 @@
       <c r="E86" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3057,12 +3425,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>i63</t>
+          <t>i59</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Households with improved food security (HDDS) (%)</t>
+          <t>Women-led agricultural groups legally registered (groups)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3072,7 +3440,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3084,12 +3457,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>i64</t>
+          <t>i60</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Hectares of degraded farmland restored (hectares)</t>
+          <t>Registered groups actively selling produce together (groups)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3100,6 +3473,11 @@
       <c r="E88" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3111,12 +3489,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>i65</t>
+          <t>i61</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Community platforms established, one per clan, engaging local authorities (platforms)</t>
+          <t>Average increase in group sales revenue (%)</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3127,84 +3505,141 @@
       <c r="E89" t="inlineStr">
         <is>
           <t>count</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>indicator</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>charles</t>
+          <t>i62</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Charles Karbedeh Jr.</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
+          <t>Average increase in household income (%)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>indicator</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>women_coord</t>
+          <t>i63</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Women's Rights Coordinator</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
+          <t>Households with improved food security (HDDS) (%)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>indicator</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>agro_coord</t>
+          <t>i64</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Agroecology Coordinator</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
+          <t>Hectares of degraded farmland restored (hectares)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>indicator</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>legal_coord</t>
+          <t>i65</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Legal Empowerment Coordinator</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
+          <t>Community platforms established, one per clan, engaging local authorities (platforms)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3214,16 +3649,97 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>women_agri_coord</t>
+          <t>charles</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Women Agricultural Resilience Coordinator</t>
+          <t>Charles Karbedeh Jr.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>women_coord</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Women's Rights Coordinator</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>agro_coord</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Agroecology Coordinator</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>legal_coord</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Legal Empowerment Coordinator</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>women_agri_coord</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Women Agricultural Resilience Coordinator</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update YALL M&E indicators and dashboard
</commit_message>
<xml_diff>
--- a/kobo/YALL_MEAL_Indicator_Update.xlsx
+++ b/kobo/YALL_MEAL_Indicator_Update.xlsx
@@ -486,11 +486,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -513,15 +508,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>project=${project}</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -544,11 +535,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -571,15 +557,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>project=${project}</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -607,10 +589,6 @@
           <t>instance('indicator')/root/item[name=${indicator}]/kind!='percent'</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -638,10 +616,6 @@
           <t>instance('indicator')/root/item[name=${indicator}]/kind='percent'</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -669,8 +643,6 @@
           <t>instance('indicator')/root/item[name=${indicator}]/kind='percent'</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>.&lt;=${assessed}</t>
@@ -708,10 +680,6 @@
           <t>instance('indicator')/root/item[name=${indicator}]/gender='yes'</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -739,10 +707,6 @@
           <t>instance('indicator')/root/item[name=${indicator}]/gender='yes'</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -765,15 +729,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>today()</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -796,11 +756,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -823,11 +778,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -850,11 +800,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -877,11 +822,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -894,7 +834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -945,9 +885,6 @@
           <t>Defending Women's Environmental and Human Rights Against Mining-Induced Degradation</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -965,9 +902,6 @@
           <t>Agroecology for Resilient Livelihoods in Mining-Affected Communities</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -985,9 +919,6 @@
           <t>Empowering Communities for Climate Justice through Legal Strategies for Safe Artisanal Mining Practices in Liberia</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1005,9 +936,6 @@
           <t>The Women Agricultural Resilience Initiative</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1030,8 +958,6 @@
           <t>uaf_women</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1054,8 +980,6 @@
           <t>uaf_women</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1078,8 +1002,6 @@
           <t>uaf_women</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1102,8 +1024,6 @@
           <t>uaf_women</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1126,8 +1046,6 @@
           <t>uaf_women</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1150,8 +1068,6 @@
           <t>uaf_women</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1174,8 +1090,6 @@
           <t>agroecology</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1198,8 +1112,6 @@
           <t>agroecology</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1222,8 +1134,6 @@
           <t>agroecology</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1246,8 +1156,6 @@
           <t>legal_empowerment</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1270,8 +1178,6 @@
           <t>legal_empowerment</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1294,8 +1200,6 @@
           <t>legal_empowerment</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1318,8 +1222,6 @@
           <t>legal_empowerment</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1342,8 +1244,6 @@
           <t>legal_empowerment</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1366,8 +1266,6 @@
           <t>legal_empowerment</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1390,8 +1288,6 @@
           <t>legal_empowerment</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1414,8 +1310,6 @@
           <t>legal_empowerment</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1438,8 +1332,6 @@
           <t>women_agri</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1462,8 +1354,6 @@
           <t>women_agri</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1486,8 +1376,6 @@
           <t>women_agri</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1510,8 +1398,6 @@
           <t>women_agri</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1534,8 +1420,6 @@
           <t>women_agri</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1558,8 +1442,6 @@
           <t>women_agri</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1569,22 +1451,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i31</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Women leaders trained in legal empowerment, water monitoring, evidence gathering (women leaders)</t>
+          <t>Formal partnership agreement signed with EPA (agreements)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1601,17 +1483,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i32</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Community dialogue sessions conducted (sessions)</t>
+          <t>Joint activities conducted with EPA (trainings, monitoring visits, compliance sessions) (activities)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1633,17 +1515,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i33</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Shadow report published (reports)</t>
+          <t>Community members trained on legal advocacy (people)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1653,7 +1535,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1665,22 +1547,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>i4</t>
+          <t>i34</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Copies of shadow report disseminated (copies)</t>
+          <t>Trained community members aware of land rights (%)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1697,22 +1579,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>i5</t>
+          <t>i35</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Advocacy meetings held with decision-makers (meetings)</t>
+          <t>Trained community members who know where to report environmental damage (%)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1729,17 +1611,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>i6</t>
+          <t>i36</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>New EPA investigations initiated from community-generated evidence (investigations)</t>
+          <t>Community members engaged in documented advocacy action post-training (people)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1749,7 +1631,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1761,17 +1643,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>i7</t>
+          <t>i37</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Agroecology demonstration plots established (plots)</t>
+          <t>Community advocacy associations (Community Advocacy Hub) formed and active (associations)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1793,17 +1675,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>i8</t>
+          <t>i38</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Women farmers trained in agroecological practices (women farmers)</t>
+          <t>Active members across community advocacy associations (at least 10 per community) (members)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1813,7 +1695,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1825,17 +1707,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>i9</t>
+          <t>i39</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Women farmers adopting at least 4 agroecological techniques (women farmers)</t>
+          <t>Advocacy actions taken by association members (at least 2 per community) (actions)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1857,17 +1739,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>i10</t>
+          <t>i40</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Radio awareness sessions aired (sessions)</t>
+          <t>Community members reached through association-led advocacy activities (people)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1877,7 +1759,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1771,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>i11</t>
+          <t>i41</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Social media content pieces produced (content pieces)</t>
+          <t>Miners trained on safe mining practices (miners)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1909,7 +1791,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1921,22 +1803,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>i12</t>
+          <t>i42</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CSOs participating in the Rural Women Climate Justice Summit (organizations)</t>
+          <t>Trained miners demonstrating improved knowledge of safety protocols (%)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1953,22 +1835,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>i13</t>
+          <t>i43</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Policy proposal tabled by coalition (proposals)</t>
+          <t>Trained miners reporting consistent PPE use at 3-month follow-up (%)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1985,22 +1867,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>i14</t>
+          <t>i44</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Organizations in the coalition tabling the policy proposal (organizations)</t>
+          <t>Trained miners aware of mining laws and regulations (%)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>uaf_women</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2017,22 +1899,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>i15</t>
+          <t>i45</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Agroecological demonstration sites established (sites)</t>
+          <t>Trained miners who fill or cover pits after mining (%)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2049,17 +1931,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>i16</t>
+          <t>i46</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Demonstration sites with soil and water conservation structures in place (sites)</t>
+          <t>Students reached through climate change workshops (the student hub ambassadors) (students)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2069,7 +1951,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2081,17 +1963,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>i17</t>
+          <t>i47</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tool sheds and storage units constructed (sheds)</t>
+          <t>Schools participating in climate change workshops (schools)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2113,27 +1995,27 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>i18</t>
+          <t>i48</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Farmers trained in climate-smart agroecological practices (farmers)</t>
+          <t>Students demonstrating improved climate change knowledge after workshops (%)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2145,22 +2027,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>i19</t>
+          <t>i50</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Female participants among trained farmers (%)</t>
+          <t>Community-led climate-sensitive projects initiated through the hub (projects)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2177,22 +2059,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>i20</t>
+          <t>i70</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Trained farmers demonstrating knowledge of at least 3 techniques (%)</t>
+          <t>Student-led climate justice initiatives implemented on campuses through the hub (initiatives)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2209,27 +2091,27 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>i21</t>
+          <t>i51</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Trained farmers adopting at least 3 new practices (%)</t>
+          <t>Community members engaged through hub activities (people)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2241,17 +2123,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>i22</t>
+          <t>i52</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Vegetable crop varieties planted and harvested (varieties)</t>
+          <t>Training manuals developed (legal advocacy, safe mining, climate change, hub management) (manuals)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2273,17 +2155,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>i23</t>
+          <t>i53</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Harvest consumed by participating households (%)</t>
+          <t>Planned training sessions delivered using the developed manuals (%)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2305,17 +2187,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>i24</t>
+          <t>i54</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Harvest sold collectively (%)</t>
+          <t>Facilitators rating the training manuals as useful or highly useful (%)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>agroecology</t>
+          <t>legal_empowerment</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2337,12 +2219,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>i25</t>
+          <t>i15</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Farmers completing agro-entrepreneurship training (farmers)</t>
+          <t>Agroecological demonstration sites established (sites)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2357,7 +2239,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2251,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>i26</t>
+          <t>i16</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Farmer groups maintaining financial records (groups)</t>
+          <t>Demonstration sites with soil and water conservation structures in place (sites)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2401,12 +2283,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>i27</t>
+          <t>i17</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Farmer groups with an active susu fund (groups)</t>
+          <t>Tool sheds and storage units constructed (sheds)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2433,12 +2315,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>i28</t>
+          <t>i18</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Increase in average household income from produce sales (%)</t>
+          <t>Farmers trained in climate-smart agroecological practices (farmers)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2453,7 +2335,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2465,12 +2347,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>i29</t>
+          <t>i19</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Farmer groups participating in final evaluation workshop (groups)</t>
+          <t>Female participants among trained farmers (%)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2480,7 +2362,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2497,12 +2379,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>i30</t>
+          <t>i20</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Written sustainability plans produced and adopted (plans)</t>
+          <t>Trained farmers demonstrating knowledge of at least 3 techniques (%)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2512,7 +2394,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2529,22 +2411,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>i31</t>
+          <t>i21</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Formal partnership agreement signed with EPA (agreements)</t>
+          <t>Trained farmers adopting at least 3 new practices (%)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2561,17 +2443,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>i32</t>
+          <t>i22</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Joint activities conducted with EPA (activities)</t>
+          <t>Vegetable crop varieties planted and harvested (varieties)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2593,27 +2475,27 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>i33</t>
+          <t>i23</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Community members trained on legal advocacy (people)</t>
+          <t>Harvest consumed by participating households (%)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2625,17 +2507,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>i34</t>
+          <t>i24</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Trained community members demonstrating improved knowledge of land rights (%)</t>
+          <t>Harvest sold collectively (%)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2657,27 +2539,27 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>i35</t>
+          <t>i25</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Trained community members who know where to report environmental damage (%)</t>
+          <t>Farmers completing agro-entrepreneurship training (farmers)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2689,17 +2571,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>i36</t>
+          <t>i26</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Community members engaged in documented advocacy action post-training (people)</t>
+          <t>Farmer groups maintaining financial records (groups)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2709,7 +2591,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2721,17 +2603,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>i37</t>
+          <t>i27</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Community advocacy associations formed and active (associations)</t>
+          <t>Farmer groups with an active susu fund (groups)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2753,27 +2635,27 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>i38</t>
+          <t>i28</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Active members across community advocacy associations (members)</t>
+          <t>Increase in average household income from produce sales (%)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>average</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2785,17 +2667,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>i39</t>
+          <t>i29</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Advocacy actions taken by association members (actions)</t>
+          <t>Farmer groups participating in final evaluation workshop (groups)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2817,17 +2699,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>i40</t>
+          <t>i30</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Community members reached through association-led advocacy activities (people)</t>
+          <t>Written sustainability plans produced and adopted (plans)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>agroecology</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2837,7 +2719,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2849,17 +2731,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>i41</t>
+          <t>i1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Miners trained on safe mining practices (miners)</t>
+          <t>Women leaders trained in legal empowerment, water monitoring, evidence gathering (women leaders)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2869,7 +2751,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -2881,22 +2763,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>i42</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Trained miners demonstrating improved knowledge of safety protocols (%)</t>
+          <t>Community dialogue sessions conducted (sessions)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -2913,22 +2795,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>i43</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Trained miners reporting consistent PPE use post-training (%)</t>
+          <t>Shadow report published (reports)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2945,22 +2827,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>i44</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Trained miners aware of mining laws and regulations (%)</t>
+          <t>Copies of shadow report disseminated (copies)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2977,22 +2859,22 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>i45</t>
+          <t>i5</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Miners who fill or cover pits after mining (%)</t>
+          <t>Advocacy meetings held with decision-makers (meetings)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3009,17 +2891,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>i46</t>
+          <t>i6</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Students reached through climate change workshops (students)</t>
+          <t>New EPA investigations initiated from community-generated evidence (investigations)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3029,7 +2911,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3041,17 +2923,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>i47</t>
+          <t>i7</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Schools participating in climate change workshops (schools)</t>
+          <t>Agroecology demonstration plots established (plots)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3073,22 +2955,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>i48</t>
+          <t>i8</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Students demonstrating improved climate change knowledge (%)</t>
+          <t>Women farmers trained in agroecological practices (women farmers)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3105,17 +2987,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>i49</t>
+          <t>i9</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Climate Justice Hub established and operational (hubs)</t>
+          <t>Women farmers adopting at least 4 agroecological techniques (women farmers)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3137,17 +3019,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>i50</t>
+          <t>i10</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Community-led climate-sensitive projects initiated through the hub (projects)</t>
+          <t>Radio awareness sessions aired (sessions)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3169,17 +3051,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>i51</t>
+          <t>i11</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Community members engaged through hub activities (people)</t>
+          <t>Social media content pieces produced (content pieces)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3189,7 +3071,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3201,17 +3083,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>i52</t>
+          <t>i12</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Training manuals developed (manuals)</t>
+          <t>CSOs, women's rights organizations and environmental justice networks participating in the Rural Women Climate Justice Summit (organizations)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3233,22 +3115,22 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>i53</t>
+          <t>i13</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Training sessions conducted using the developed manuals (%)</t>
+          <t>Policy proposal on environmental and land tenure clauses in mining concession agreements tabled by the coalition (proposals)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3265,22 +3147,22 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>i54</t>
+          <t>i14</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Facilitators rating the training manuals as useful or highly useful (%)</t>
+          <t>Community-based CSOs in the coalition tabling the policy proposal (organizations)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>legal_empowerment</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3297,17 +3179,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>i55</t>
+          <t>i66</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Women farmers participating in training (women farmers)</t>
+          <t>EPA investigations with initial findings publicly reported (investigations)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3329,22 +3211,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>i56</t>
+          <t>i67</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Women farmers who know at least 3 climate-smart techniques (%)</t>
+          <t>Evidence submissions (water test results, photo and video documentation, testimonies) by trained women leaders to the EPA (at least 2 per community) (submissions)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3361,17 +3243,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>i57</t>
+          <t>i68</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Women farmers applying at least 3 techniques on their farms (%)</t>
+          <t>Adopting women farmers reporting improved soil health and crop diversity and growth (%)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3393,22 +3275,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>i58</t>
+          <t>i69</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Average crop yield increase (%)</t>
+          <t>Adopting women farmers reporting improved food security and economic independence (%)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>women_agri</t>
+          <t>uaf_women</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3425,12 +3307,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>i59</t>
+          <t>i55</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Women-led agricultural groups legally registered (groups)</t>
+          <t>Women farmers participating in training (women farmers)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3457,12 +3339,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>i60</t>
+          <t>i56</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Registered groups actively selling produce together (groups)</t>
+          <t>Trained women farmers who know at least 3 climate-smart techniques (%)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3472,7 +3354,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3489,12 +3371,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>i61</t>
+          <t>i57</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Average increase in group sales revenue (%)</t>
+          <t>Trained women farmers applying at least 3 techniques on their farms (%)</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3504,7 +3386,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3521,12 +3403,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>i62</t>
+          <t>i58</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Average increase in household income (%)</t>
+          <t>Average crop yield increase (%)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3536,7 +3418,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>average</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3553,12 +3435,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>i63</t>
+          <t>i59</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Households with improved food security (HDDS) (%)</t>
+          <t>Women-led agricultural groups legally registered (by end of project) (groups)</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3568,7 +3450,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>count</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3585,12 +3467,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>i64</t>
+          <t>i60</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Hectares of degraded farmland restored (hectares)</t>
+          <t>Registered groups actively selling produce together (groups)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3617,12 +3499,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>i65</t>
+          <t>i61</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Community platforms established, one per clan, engaging local authorities (platforms)</t>
+          <t>Average increase in group sales revenue (%)</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3632,7 +3514,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>average</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3644,102 +3526,279 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>indicator</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>charles</t>
+          <t>i62</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Charles Karbedeh Jr.</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr"/>
+          <t>Average increase in household income (%)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>average</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>indicator</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>women_coord</t>
+          <t>i63</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Women's Rights Coordinator</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
+          <t>Women-headed households facing severe food insecurity (measured by HDDS) (%)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>indicator</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>agro_coord</t>
+          <t>i64</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Agroecology Coordinator</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
+          <t>Hectares of degraded farmland restored (hectares)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>indicator</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>legal_coord</t>
+          <t>i65</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Legal Empowerment Coordinator</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
+          <t>Community platforms established, one per clan, engaging local authorities on land rights and environmental protection (platforms)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
+          <t>indicator</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>i71</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Women-led agricultural groups that are financially literate (groups)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>indicator</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>i72</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Community platforms with women leaders in key roles (platforms)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>women_agri</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>coordinator</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>charles</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Charles Karbedeh Jr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>women_coord</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Women's Rights Coordinator</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>agro_coord</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Agroecology Coordinator</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>legal_coord</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Legal Empowerment Coordinator</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
         <is>
           <t>women_agri_coord</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>Women Agricultural Resilience Coordinator</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>